<commit_message>
added workflow 3 documentation
</commit_message>
<xml_diff>
--- a/doc/evaluation.xlsx
+++ b/doc/evaluation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\FH\4.Semester\KIS4\projekt-bb-g2-pointner-kaltenegger\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF0503BC-137F-4417-BEAB-6B095EDB6FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D5DEE23-8B2A-4387-A1D2-BD76A24D1E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="3" xr2:uid="{13E085B4-8549-4F7A-A15F-5AE90E5F5FCC}"/>
+    <workbookView xWindow="-180" yWindow="-180" windowWidth="38760" windowHeight="21240" activeTab="3" xr2:uid="{13E085B4-8549-4F7A-A15F-5AE90E5F5FCC}"/>
   </bookViews>
   <sheets>
     <sheet name="Tokenverbrauch" sheetId="2" r:id="rId1"/>
@@ -260,9 +260,8 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -273,15 +272,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1">
       <extLst>
@@ -290,9 +283,6 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1">
       <extLst>
@@ -300,9 +290,6 @@
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1">
@@ -314,6 +301,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Ausgabe" xfId="2" builtinId="21"/>
@@ -428,6 +427,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-8E91-4B12-B137-CCDA22E11244}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -447,6 +451,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-8E91-4B12-B137-CCDA22E11244}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -466,6 +475,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-8E91-4B12-B137-CCDA22E11244}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -543,13 +557,13 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.16666666666666666</c:v>
+                  <c:v>4.8393341076267905E-5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.33333333333333331</c:v>
+                  <c:v>9.6786682152535811E-5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.5</c:v>
+                  <c:v>0.99985481997677117</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -734,7 +748,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="de-DE"/>
+          <a:endParaRPr lang="de-AT"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -853,7 +867,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -972,7 +986,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1091,7 +1105,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1419,7 +1433,7 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1707,7 +1721,7 @@
                   <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4604,76 +4618,76 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>1</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>2</v>
       </c>
-      <c r="D3" s="10">
-        <v>3</v>
+      <c r="D3" s="8">
+        <v>15784</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="9">
         <v>0</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="9">
         <v>0</v>
       </c>
-      <c r="D4" s="11">
-        <v>0</v>
+      <c r="D4" s="9">
+        <v>4877</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="16">
         <v>0</v>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="16">
         <v>0</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="16">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="17">
         <f>SUM(B3:B5)</f>
         <v>1</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="17">
         <f t="shared" ref="C6:D6" si="0">SUM(C3:C5)</f>
         <v>2</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="17">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>20661</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -4682,34 +4696,34 @@
       </c>
       <c r="B8">
         <f>SUM(B6:D6)</f>
-        <v>6</v>
+        <v>20664</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <f>B6/B8</f>
-        <v>0.16666666666666666</v>
+        <v>4.8393341076267905E-5</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <f>C6/B8</f>
-        <v>0.33333333333333331</v>
+        <v>9.6786682152535811E-5</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <f>D6/B8</f>
-        <v>0.5</v>
+        <v>0.99985481997677117</v>
       </c>
     </row>
   </sheetData>
@@ -4729,268 +4743,268 @@
   </cols>
   <sheetData>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" t="s">
         <v>0</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="14" t="b">
+      <c r="C13" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="D13" s="14" t="b">
+      <c r="D13" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="14" t="b">
-        <v>0</v>
+      <c r="E13" s="11" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="13" t="s">
+      <c r="A14" s="20"/>
+      <c r="B14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="14" t="b">
+      <c r="C14" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="D14" s="14" t="b">
+      <c r="D14" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="14" t="b">
-        <v>0</v>
+      <c r="E14" s="11" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
-      <c r="B15" s="13" t="s">
+      <c r="A15" s="20"/>
+      <c r="B15" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="14" t="b">
+      <c r="C15" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="D15" s="14" t="b">
+      <c r="D15" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="14" t="b">
-        <v>0</v>
+      <c r="E15" s="11" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="12"/>
-      <c r="B16" s="13" t="s">
+      <c r="A16" s="20"/>
+      <c r="B16" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="14" t="b">
+      <c r="C16" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="D16" s="14" t="b">
+      <c r="D16" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="14" t="b">
-        <v>0</v>
+      <c r="E16" s="11" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3" t="s">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="3">
         <f>(C13+C14+C15+C16) / 4</f>
         <v>0</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <f t="shared" ref="D17:E17" si="0">(D13+D14+D15+D16) / 4</f>
         <v>0</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="17" t="b">
+      <c r="C18" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="D18" s="17" t="b">
+      <c r="D18" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="17" t="b">
-        <v>0</v>
+      <c r="E18" s="13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16" t="s">
+      <c r="A19" s="21"/>
+      <c r="B19" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="17" t="b">
+      <c r="C19" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="D19" s="17" t="b">
+      <c r="D19" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="17" t="b">
-        <v>0</v>
+      <c r="E19" s="13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="15"/>
-      <c r="B20" s="16" t="s">
+      <c r="A20" s="21"/>
+      <c r="B20" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="17" t="b">
+      <c r="C20" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="D20" s="17" t="b">
+      <c r="D20" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="17" t="b">
-        <v>0</v>
+      <c r="E20" s="13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3" t="s">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="3">
         <f>(C18+C19+C20) / 3</f>
         <v>0</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="3">
         <f t="shared" ref="D21:E21" si="1">(D18+D19+D20) / 3</f>
         <v>0</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C22" s="20" t="b">
+      <c r="C22" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="D22" s="20" t="b">
+      <c r="D22" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="20" t="b">
-        <v>0</v>
+      <c r="E22" s="15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="18"/>
-      <c r="B23" s="19" t="s">
+      <c r="A23" s="19"/>
+      <c r="B23" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C23" s="20" t="b">
+      <c r="C23" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="D23" s="20" t="b">
+      <c r="D23" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="20" t="b">
-        <v>0</v>
+      <c r="E23" s="15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="18"/>
-      <c r="B24" s="19" t="s">
+      <c r="A24" s="19"/>
+      <c r="B24" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C24" s="20" t="b">
+      <c r="C24" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="D24" s="20" t="b">
+      <c r="D24" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="20" t="b">
-        <v>0</v>
+      <c r="E24" s="15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3" t="s">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="3">
         <f>(C22+C23+C24) / 3</f>
         <v>0</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="3">
         <f t="shared" ref="D25" si="2">(D22+D23+D24) / 3</f>
         <v>0</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="3">
         <f t="shared" ref="E25" si="3">(E22+E23+E24) / 3</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5" t="s">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="5">
         <f>(C17+C21+C25) / 3</f>
         <v>0</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="5">
         <f t="shared" ref="D26:E26" si="4">(D17+D21+D25) / 3</f>
         <v>0</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="5">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>21</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>9</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" t="s">
         <v>0</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D31" t="s">
         <v>1</v>
       </c>
     </row>
@@ -4998,51 +5012,51 @@
       <c r="A32" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="7">
         <f>C17 / 3</f>
         <v>0</v>
       </c>
-      <c r="C32" s="9">
+      <c r="C32" s="7">
         <f t="shared" ref="C32:D32" si="5">D17 / 3</f>
         <v>0</v>
       </c>
-      <c r="D32" s="9">
+      <c r="D32" s="7">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="9">
+      <c r="B33" s="7">
         <f>C21 / 3</f>
         <v>0</v>
       </c>
-      <c r="C33" s="9">
+      <c r="C33" s="7">
         <f t="shared" ref="C33:D33" si="6">D21 / 3</f>
         <v>0</v>
       </c>
-      <c r="D33" s="9">
+      <c r="D33" s="7">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>18</v>
       </c>
-      <c r="B34" s="9">
+      <c r="B34" s="7">
         <f>C25 / 3</f>
         <v>0</v>
       </c>
-      <c r="C34" s="9">
+      <c r="C34" s="7">
         <f t="shared" ref="C34:D34" si="7">D25 / 3</f>
         <v>0</v>
       </c>
-      <c r="D34" s="9">
+      <c r="D34" s="7">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
     </row>
   </sheetData>
@@ -5088,7 +5102,7 @@
         <v>2</v>
       </c>
       <c r="D3">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -5130,7 +5144,7 @@
         <v>3</v>
       </c>
       <c r="D4">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>